<commit_message>
Otimizando o filtro e o processamento dos dados
</commit_message>
<xml_diff>
--- a/spreadsheets/clean_structured_data/clean_structured_data.xlsx
+++ b/spreadsheets/clean_structured_data/clean_structured_data.xlsx
@@ -16,10 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -58,12 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -576,8 +572,10 @@
       <c r="N2" t="n">
         <v>5</v>
       </c>
-      <c r="O2" s="2" t="n">
-        <v>47837</v>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>20/12/2030</t>
+        </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -593,16 +591,24 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LCI BANCO FULANO - DEZ/2030</t>
+          <t>LCI BANCO CICLANO - DEZ/2030</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Digital</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>96,5% CDI</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>108,675% CDI</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>LCI</t>
@@ -639,8 +645,10 @@
       <c r="N3" t="n">
         <v>5</v>
       </c>
-      <c r="O3" s="2" t="n">
-        <v>47837</v>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>20/12/2030</t>
+        </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -656,15 +664,19 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LCI BANCO FULANO - DEZ/2030</t>
+          <t>LCI BANCO CICLANO - DEZ/2030</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Exclusive</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>Digital</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>93% CDI</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
@@ -702,8 +714,10 @@
       <c r="N4" t="n">
         <v>5</v>
       </c>
-      <c r="O4" s="2" t="n">
-        <v>47837</v>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>20/12/2030</t>
+        </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -719,15 +733,19 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LCI BANCO FULANO - DEZ/2030</t>
+          <t>LCI BANCO CICLANO - DEZ/2030</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>Exclusive</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>94% CDI</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
@@ -765,8 +783,10 @@
       <c r="N5" t="n">
         <v>5</v>
       </c>
-      <c r="O5" s="2" t="n">
-        <v>47837</v>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>20/12/2030</t>
+        </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -782,15 +802,19 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LCI BANCO FULANO - DEZ/2030</t>
+          <t>LCI BANCO CICLANO - DEZ/2030</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Unique</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>95% CDI</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
@@ -828,8 +852,10 @@
       <c r="N6" t="n">
         <v>5</v>
       </c>
-      <c r="O6" s="2" t="n">
-        <v>47837</v>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>20/12/2030</t>
+        </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -845,15 +871,19 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LCI BANCO FULANO - DEZ/2030</t>
+          <t>LCI BANCO CICLANO - DEZ/2030</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>96,5% CDI</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
@@ -891,8 +921,10 @@
       <c r="N7" t="n">
         <v>5</v>
       </c>
-      <c r="O7" s="2" t="n">
-        <v>47837</v>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>20/12/2030</t>
+        </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
@@ -913,7 +945,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -921,11 +953,7 @@
           <t>96,5% CDI</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>108,675% CDI</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>LCI</t>
@@ -962,8 +990,10 @@
       <c r="N8" t="n">
         <v>5</v>
       </c>
-      <c r="O8" s="2" t="n">
-        <v>47837</v>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>20/12/2030</t>
+        </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
@@ -971,341 +1001,6 @@
         </is>
       </c>
       <c r="Q8" t="inlineStr">
-        <is>
-          <t>Investidor Geral</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>LCI BANCO CICLANO - DEZ/2030</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Digital</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>93% CDI</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>LCI</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>LETRA DE CRÉDITO IMOBILIÁRIO</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>% CDI</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="N9" t="n">
-        <v>5</v>
-      </c>
-      <c r="O9" s="2" t="n">
-        <v>47837</v>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>1,21%</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>Investidor Geral</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>LCI BANCO CICLANO - DEZ/2030</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Exclusive</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>94% CDI</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>LCI</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>LETRA DE CRÉDITO IMOBILIÁRIO</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>% CDI</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="N10" t="n">
-        <v>5</v>
-      </c>
-      <c r="O10" s="2" t="n">
-        <v>47837</v>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>1,21%</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>Investidor Geral</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>LCI BANCO CICLANO - DEZ/2030</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>95% CDI</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>LCI</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>LETRA DE CRÉDITO IMOBILIÁRIO</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>% CDI</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="N11" t="n">
-        <v>5</v>
-      </c>
-      <c r="O11" s="2" t="n">
-        <v>47837</v>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>1,21%</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>Investidor Geral</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>LCI BANCO CICLANO - DEZ/2030</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Unique</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>96,5% CDI</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>LCI</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>LETRA DE CRÉDITO IMOBILIÁRIO</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>% CDI</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="N12" t="n">
-        <v>5</v>
-      </c>
-      <c r="O12" s="2" t="n">
-        <v>47837</v>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>1,21%</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>Investidor Geral</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>LCI BANCO CICLANO - DEZ/2030</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>96,5% CDI</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>LCI</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>LETRA DE CRÉDITO IMOBILIÁRIO</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>% CDI</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="N13" t="n">
-        <v>5</v>
-      </c>
-      <c r="O13" s="2" t="n">
-        <v>47837</v>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>1,21%</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
         <is>
           <t>Investidor Geral</t>
         </is>

</xml_diff>

<commit_message>
Adicionando o tratamente de produtos segmentados
</commit_message>
<xml_diff>
--- a/spreadsheets/clean_structured_data/clean_structured_data.xlsx
+++ b/spreadsheets/clean_structured_data/clean_structured_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -596,17 +596,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Digital</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>96,5% CDI</t>
+          <t>93% CDI</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>108,675% CDI</t>
+          <t>102% CDI</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -669,15 +669,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Digital</t>
+          <t>Exclusive</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>93% CDI</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>94% CDI</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>103% CDI</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>LCI</t>
@@ -738,15 +742,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Exclusive</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>94% CDI</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>95% CDI</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>104% CDI</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>LCI</t>
@@ -807,15 +815,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Signature</t>
+          <t>Unique</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>95% CDI</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>96,5% CDI</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>105% CDI</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>LCI</t>
@@ -876,7 +888,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -884,7 +896,11 @@
           <t>96,5% CDI</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>106% CDI</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>LCI</t>
@@ -932,75 +948,6 @@
         </is>
       </c>
       <c r="Q7" t="inlineStr">
-        <is>
-          <t>Investidor Geral</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>LCI BANCO CICLANO - DEZ/2030</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>96,5% CDI</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>LCI</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>LETRA DE CRÉDITO IMOBILIÁRIO</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>% CDI</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="N8" t="n">
-        <v>5</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>20/12/2030</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>1,21%</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
         <is>
           <t>Investidor Geral</t>
         </is>

</xml_diff>